<commit_message>
Reset DB and MIN_CODEs to current state (Video 6342, Audio 1254)
</commit_message>
<xml_diff>
--- a/settings.xlsx
+++ b/settings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,476 +436,2788 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>savam45676@daikoa.com</t>
+          <t>daret35933@nctime.com</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>76wdvssqe4Z5TW2prOzqjNKS1X0JddFq</t>
+          <t>gTRZleGLlpRXuN4JR3Z69urgNhvfZgXf</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ermjT6fUpjdwJ8Cpbaop8R</t>
+          <t>uGK7YELaKdSF9gf9ATmXoX</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>wogero4961@dretnar.com</t>
+          <t>tafolel838@ametitas.com</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>vcGKMj18D1DDq4TS3gOEF4LOLGT2x7yQ</t>
+          <t>sTvcFcGH4S39pACPSwYXTGDhM2BEL3kP</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Bun4v3nU64AhjzpdSWiemS</t>
+          <t>KFTmYXUqypFR6JbJy7r72g</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>titow54942@dretnar.com</t>
+          <t>sekeber866@dropeso.com</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>4L16RFGlrDsOcHbpkBzt8DmJx3c20div</t>
+          <t>6m6Boofi3vyiye1mWGk2z8JPLedRYP1l</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>wMo7tcJSzPFdqVVwkdkhSF</t>
+          <t>mqhhwkNjs6LbnusE87WgxF</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>povej18527@dretnar.com</t>
+          <t>fatisis252@filipx.com</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Wb2hayUo3xugCXuNWIIJdTGEsY17ZKdK</t>
+          <t>xXM7YgF9EfC9ObxBpbjd3oUxmIDj0E1J</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>hVxPZa2jdmwGHVj8An5hAK</t>
+          <t>H9k4tH57H8Qx2xxkDgw6ZJ</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>goyaja1050@daikoa.com</t>
+          <t>xaxaveb930@gamepec.com</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>dYiibSMdcXTcy5lDePf5nXegvIAJMtUe</t>
+          <t>Lm3LOfqVcTHWIgPEXPokowvo21CayIGZ</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>hqLMkRc27w7vg5CTSWwWmn</t>
+          <t>oJkWc6d7ikC8p8z5VRMZii</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>bocowa9157@daikoa.com</t>
+          <t>socamog235@gamepec.com</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>exrLCAXboHaXet9OlqJAN96OmKWsDnfo</t>
+          <t>80M9YjLNMMpnHxvn77VqlwjOoygXqTJJ</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>hW8WWpTLfpm69rNgikkLBY</t>
+          <t>mxPwz4s5mtD9TAxE6AkNeb</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>lokos77574@coswz.com</t>
+          <t>rerob43025@gamepec.com</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>rNU7s0xkwJcc3DDFI9osfwRqVJB5MUvd</t>
+          <t>GWODyKNPNpFbbugHbLAexY9EO4QfQgPN</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>777awg7nDxL7oVL4duMc6h</t>
+          <t>uKzUdj8mUViiqMpRne6qse</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>nojex76241@1200b.com</t>
+          <t>wonagay313@httpsu.com</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Kz7OdwkMZTZaDJQ1iUTZLbGvoS84keOP</t>
+          <t>JvazbN1rE4hVvXvj8QcyNGzf9sg5Xmxk</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>hVpkXzmpNbzDE5fFtiJbc2</t>
+          <t>9Tkxna4xBVXypXC4Z9TdHB</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>hovifim988@1200b.com</t>
+          <t>figalab281@idwager.com</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CK0Wp6WKiFD7acjl10G8vysxWR48wZRg</t>
+          <t>Xw4UIPg7EoCNOkbQF4LFxF1ixbErLtBU</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>P5XJ2dTaNUHsMkCoMgVS8i</t>
+          <t>jvMnLJVUmZrnt6uGnpArES</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>yawoc12567@coswz.com</t>
+          <t>rinepo9302@idwager.com</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>uT6UL7Qo9WWZFIw6nFihvEoPsRuWB2cB</t>
+          <t>sE3j0F88W18qS6xZegJpw9dYUlLOQwF8</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>J8JUeTV2yxn9wmuA5vLnfW</t>
+          <t>HXjPdNqjJZbmLYnUajk8Nf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>gecadac197@coswz.com</t>
+          <t>hoboxo4549@httpsu.com</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Grzwxyx41AkWP5m4f3xtEu0JlfrFim7P</t>
+          <t>OuWxiJIp9xmP2fopYIDPJgXuV6gC7g5R</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SARbUSMkNZD9XjpwUeK4oH</t>
+          <t xml:space="preserve"> y4BhwAH4FDg4cC8QQHDVKB</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>goyixov775@1200b.com</t>
+          <t>xefes61540@httpsu.com</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>h6VvXzCUwwTE11bRqNCZS8brKBY5zCbz</t>
+          <t>1YEdnC1nUvGW7P1hEGehAs8os2fzoEhp</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>REZRkCf7tSD37FJmyWRET3</t>
+          <t>n38HSjtVqUzK4bLNXgg9wA</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>jayit97735@1200b.com</t>
+          <t>dipah74837@httpsu.com</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>xstn0Y1QeBj5bnDGrXeOn648TCmCcc0G</t>
+          <t>NlidtI9aaO82ajLNo7AryVWkMNYeItXd</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>9LJtRkXV4MTjAwMVwgoUaf</t>
+          <t>ZTXVi2xiJJzSLNRe4yxeX2</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>bawavip104@coswz.com</t>
+          <t>nawat37231@roastic.com</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>JtZpye7pdPl6lK7UTCMhuZoY2hvyJ9pK</t>
+          <t>FdXCpc87a5uQhVaqntEyZzjryF5rlACw</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>mTJtCxtdppM3YpyJcQDFkS</t>
+          <t>ycGayRsKw7WvUeSsMdjz5Q</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>copawo7293@coswz.com</t>
+          <t>varaf33883@naqulu.com</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>B0Mc8vRk33LEEYPIhYNJ6GOBTsBtC7Kx</t>
+          <t>531lLSFzKRS2pMW7R6AjQyoYg0nJfSfQ</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>yNVgoudEmCGXPJy5TKYFuJ</t>
+          <t>i7H4EWbcteZc93wmisovt4</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>yociko1703@1200b.com</t>
+          <t>fetip10878@roastic.com</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Uu7qo08f3qrpYeZGiovbd4b6fMvJpg5T</t>
+          <t>7SZJWYq9ZbsEnQiZ7J2NapfHWz6q5z39</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>w4bB4KNZafhZtw8Dv7Vq7c</t>
+          <t>bJCYMBgi9ifri7qi8HFWy3</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>yohiho1186@1200b.com</t>
+          <t>hexori1127@roastic.com</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>y1ROvKdGD3IfK2LpQJ6emLeiryUyeTOy</t>
+          <t>oNV0c2SijXp7CxRlzuqivcRZ3wo5VZBf</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>U3eNhDLmBZ9kbbgQuTJggg</t>
+          <t>wyW6Rqxu8K8TYkgVPsKeKn</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>vepek51758@coswz.com</t>
+          <t>linide1021@roastic.com</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Xd0XnvFWpuYJb6EyX4v0qZGJyzKPbpjf</t>
+          <t>ZeVGmMKpmGC4OZjycckcVFyijfXwHksS</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>K7wD42ADsf3yKih2DpdZX3</t>
+          <t>2oPnuNvyrRsUbQMuRq9oVA</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>vicexa9591@coswz.com</t>
+          <t>licav42884@naqulu.com</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>npz20JjzNH92wIH4tCQx49nC0it14Xxw</t>
+          <t>hnL1dYZNWM8b8MEWTHA6CKsNWjvxkT5D</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>rZd7CALt2MZEMHmpDtGQxB</t>
+          <t>vm8ggtLTbzzcBRMr3MGRVc</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>hecab14854@1200b.com</t>
+          <t>gopev53591@okcdeals.com</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>K8wwgIDz5G56KxRoP7JgMK2PO7C2UzvN</t>
+          <t>I0Z17qFrx7c995zbgVrqLtMM0Y6dd3h9</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>4KT5DztHkEUnCgYrNhRx4e</t>
+          <t>JgjHU3eCEeDCuM2B86evam</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>carexan555@coswz.com</t>
+          <t>dohojev953@nctime.com</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>cBLSH97sWXVnfO4kUKBNbM8eYNZcanHx</t>
+          <t>7C3qfKLEE02rUw9YCXynmrGxNPCdtKuc</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>HW37WS2fucmm8m6ZUSMU7Q</t>
+          <t>HMq3qgxGHux8TjvJGPRKMg</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>lokos77574@coswz.com</t>
+          <t>yamocot925@nctime.com</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>rNU7s0xkwJcc3DDFI9osfwRqVJB5MUvd</t>
+          <t>wht7NqRuiTvgrqaJpsxTVXxyXRnPRLDu</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>777awg7nDxL7oVL4duMc6h</t>
+          <t>rrXyG64aA6K434NmqnBkok</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>nojex76241@1200b.com</t>
+          <t>widivav664@nctime.com</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Kz7OdwkMZTZaDJQ1iUTZLbGvoS84keOP</t>
+          <t>myAJcAFPf3e7OE0ESDmS5qqHoEpqPhda</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>hVpkXzmpNbzDE5fFtiJbc2</t>
+          <t>fhAoCcEiijeJi3rtgDuNNd</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>hovifim988@1200b.com</t>
+          <t>gebasi3686@nctime.com</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CK0Wp6WKiFD7acjl10G8vysxWR48wZRg</t>
+          <t>RB9t58YEm0itLBhHXspWtsx9qsB6DB9e</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>P5XJ2dTaNUHsMkCoMgVS8i</t>
+          <t>Re4Gua6CJgPQvGKHyWtbFn</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>yawoc12567@coswz.com</t>
+          <t>racirop308@roratu.com</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>uT6UL7Qo9WWZFIw6nFihvEoPsRuWB2cB</t>
+          <t>Fp9aCSPL3V5biVE0mZDCJJHY6GDBDILv</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>J8JUeTV2yxn9wmuA5vLnfW</t>
+          <t>FnytnEAHavuLvStPGYoMAg</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>gecadac197@coswz.com</t>
+          <t>kilov89341@nctime.com</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Grzwxyx41AkWP5m4f3xtEu0JlfrFim7P</t>
+          <t>Sr9kw7c7zNpGtvhRS0MLO9H8npfMegLZ</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>SARbUSMkNZD9XjpwUeK4oH</t>
+          <t>4dYrE6SS5dSxt5qwTvzTVT</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>goyixov775@1200b.com</t>
+          <t>gevel44383@nctime.com</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>h6VvXzCUwwTE11bRqNCZS8brKBY5zCbz</t>
+          <t>bwyzzEVRYYttA7tmYbgsy4xcw7UVgV8O</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>REZRkCf7tSD37FJmyWRET3</t>
+          <t>HzPXvuSXXQ6S7iCQmMeF9T</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>fixes12536@nctime.com</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>tLFSJBbymOOz3JjD6B8Za7wIo9b5reiE</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>xuqgf72emBu6atQU9KJPwC</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>goyima8506@nctime.com</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>g7H4uFMeYmfFQlN0y5i2GvHrqHojlJ1n</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>gXDsBP9zWswMC32WWBWfAj</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>nekidi7850@roratu.com</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>MC0690dIR7s41wFmAsVT84JN5gGRF4Q8</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>zrV8izMTZxKtZeUdkketVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>wofetef124@jparksky.com</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>bNv5oiinBiebNL2MPIq8hGZx3CXVH0jm</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>hPBtQoQTuyiDLzW27UVAbE</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>daseso2631@jparksky.com</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>DRXjVQctFOWz1cQcUQODfryiXg31FjiL</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>MtHkkP5Qk2RR9zVA5gLgy9</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ririwa4119@ixospace.com</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>mcByeqm6xZDW1STLVQ8tmtMWVD4OZ0vq</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>NkaahaDx6Umohs8fhs3x7d</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>neloc13413@akixpres.com</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>5tn4iP1EdUCal3f7dlInF9hcZRWoDDam</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>dHpjvBPUa5g8Ka5MQu8A34</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>cadol56750@atinjo.com</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>JAvZf5v9odlVKpCQm04PEJIp9Qlma8be</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Dw7R7kP9dU9R5dw2ACuYee</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>gigij73348@akixpres.com</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>6uBAE8WK2oNHLqUP1scuIX5dvPgqkk6W</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>XiYeYgHxXcnH2tbqEBxtnk</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>hipota9018@atinjo.com</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>LxXoRVMl9zQRFnQ28SrktX3U2GyHcOOh</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Fx7zZF5qibuBBHkUGq6xpC</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>gigemi1270@atinjo.com</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>rsmqBLdT1vuYrCZ9rNoOuXVzZHSi6IVL</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>WKZzU8yHMSTUMeJKtNCB9W</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>veyorox418@akixpres.com</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>elL3annwEMcNszO8xI31nd9akdmbMfut</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>bJxx8YodEXUUTKXaNmTN3Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>wahesen320@atinjo.com</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Q15kREigAFjMZLUAyW1QftIpkSUpm3Zx</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Zs9EHCcnZyWv3X6iCBbiaQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>bagabe8853@atinjo.com</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>0bAH8FOjsLlu1jeIoirXHcN3hmXZ9Ll7</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>m9uGnynHJsabaD2Pyzyenn</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>riwag56154@akixpres.com</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>SnxsC4IIztaAh8Qk0WXFN6qDc4WFf9DO</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Qv3KsYMDxnp7thHQHZNfPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>wepol47565@akixpres.com</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>qw1WKJ4bDDImTMqzZi9eXLwHHkQpTSO6</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>CxXPjugqjFd6CAAuf8HZaV</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>solego9606@atinjo.com</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>9gDLSKh98F9c2SSUvuJSAr6MszvcTTLi</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>NrJch3iCXMJM9JLFxymFtg</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>wafile9558@akixpres.com</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>8tjVlDYXKoiKA9LiMXOL0Pjypq1xvhiY</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>wYwfXdMpdgViJvhHhNePnd</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>ratad81098@atinjo.com</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>0YdxGb2ITKezrGWiFa9cn7k4jOpQgO8c</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>myUuzuxSbiP7xdYD6mSd4K</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>yataven591@atinjo.com</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>ozoo16Bl6Q3dPwhmbTdvYncz362cRwXP</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>RuVixv8g3X98fMcL9cDqRV</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>noder31454@akixpres.com</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>5wR46xR4wULRGza81qbyC3Dux2fCm4RK</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>yrnwYNcvGrUNj4rKmm2svH</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>boleg64834@atinjo.com</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>WfrxUSz3OnBtuoVSpin6wSQbymWavST2</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>DuwptNFqTjaNPX9dH7ban7</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>kisagiw989@akixpres.com</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>xM16sQ7DLf5h2ELiGcc5ZeEeZr7G5liw</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>MY5dmNN2Wj95atQyKcRWtD</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>jehego4595@atinjo.com</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>nFC0pqugt0SvyHWfFImqKozyvuIASodz</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>eoxChE5ZREvYNCZkZr2xF5</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>dexexed273@atinjo.com</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>4sEBwF29AkejGdLQ7cNm4V46UrtlZL51</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>tqS5U8xzqPKuDatqWxTDAe</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>reloriv513@akixpres.com</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>0BAbfCRMLqLnNR0SGk1zdCfIDpU68ozw</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>8ziLdQSvxoHJFBm7bqx8gK</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>lejepas261@akixpres.com</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1H9QUd3bfLCMmPXprcuq6oA6P0cZZuOi</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>FrF9e7kRqvwzk8QZzucCrB</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>jegosi2800@atinjo.com</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>pRQrdbkcm8eTsnecHWkvzCDhcxlN0zgo</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>RYdSN2H3oa9uobCLnUWGrN</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>naxelaf699@akixpres.com</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>HLhpdosj0jR6TKxbcXXsZyesgfGf1AUt</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>gUM4qvu9Yvo94aDx7ZsyS6</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>yewewod514@akixpres.com</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>HsP1XnIRh2vmG847Ps4LhmL2XHHMtuf8</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>JATjdyhEfXsitwrsdw4UaP</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>secotot918@akixpres.com</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>6wHZfUI3LUTYbuTpmKSvHdtVj3zTsU6E</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>kS8op9jKuQk6RS8wHZGDUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>micis44451@atinjo.com</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>fDRR3GWUvhnQQxW0yZSu2xwBMggGBylV</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>yMJ57L5SAmDiAFHoMv2wUB</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>banode7154@daikoa.com</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>JCOSpFLRw8eGUdGUPalob9DnXs14cDFu</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>CYzAi4iqRtq9Lp8iYQVYDG</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>yelar54822@daikoa.com</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>s6JOCcXKLapyRPCZ0K7kcCTu8zRVIh6P</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>s4KF4kgtwvwqzNAETSBkEn</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>gibino1422@dretnar.com</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>nxTKC2GLECZuRdJqNxWu4FueMG6FCSss</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>wFCv2kwYEyRRBTQRWZDmWG</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>tinowa6684@dretnar.com</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>u5QKv1tzXgAuwkwmGeUdosXqJf3YE0mk</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>e6F7bArFz3xqHiyA48e7gm</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>jagala5779@daikoa.com</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>n6GPL2AghujKGoKXYFa1mDpLAN41tI8t</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>T84oseSmPvmfZjUHVnLRtK</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>dadac39765@daikoa.com</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>hldYhwMOTTzCd0VN4MiWv4PwtioXkbQD</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>SoT9i7shyBEoBsq9pdhBFS</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>xavimi2919@daikoa.com</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>D6u5oKva8hquabzZuKEYRTRmYmn4fzlK</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>7TvAhBKSBeTnapk3QYeVxG</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>savam45676@daikoa.com</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>76wdvssqe4Z5TW2prOzqjNKS1X0JddFq</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>ermjT6fUpjdwJ8Cpbaop8R</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>wogero4961@dretnar.com</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>vcGKMj18D1DDq4TS3gOEF4LOLGT2x7yQ</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Bun4v3nU64AhjzpdSWiemS</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>titow54942@dretnar.com</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>4L16RFGlrDsOcHbpkBzt8DmJx3c20div</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>wMo7tcJSzPFdqVVwkdkhSF</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>povej18527@dretnar.com</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Wb2hayUo3xugCXuNWIIJdTGEsY17ZKdK</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>hVxPZa2jdmwGHVj8An5hAK</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>goyaja1050@daikoa.com</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>dYiibSMdcXTcy5lDePf5nXegvIAJMtUe</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>hqLMkRc27w7vg5CTSWwWmn</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>bocowa9157@daikoa.com</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>exrLCAXboHaXet9OlqJAN96OmKWsDnfo</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>hW8WWpTLfpm69rNgikkLBY</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>socas91504@dretnar.com</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>zwwI8F0DewAZat1DNGEX9FDV9XrfYwfY</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>2zQjp5rCLonb2UqmPNiwf5</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>milidij455@dretnar.com</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>HfekRAMQdJuiL1IyQ2LU7Gf55ek6NEKr</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>spQpD2WBbZirL7UNvRrpNA</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>lipota2474@1200b.com</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>UKAWL111GeXpmJxRG6ijnrUrXau0TQWe</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>ay2xrft7cY3VC928BPUacE</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>gidevok422@1200b.com</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>DtSxMlHMagZAFQHV5WiiaNI9bmqg2UkQ</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>NREwQMq757tnLqK3U5WoPV</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>tofepi1509@coswz.com</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>K2qGEA8d2aRQm4p4RVVHdfWw16i1vLHb</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>7BoB84re8TsrnpfpmY5Xg7</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>hejita4492@coswz.com</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>3lFTo0Rnbv9YiWfy3gO5xjwfHXPYNa4A</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>zXCFEZncTGyiQ2gaMi8fpm</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>doxixi5794@1200b.com</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>J6q60nEZvsFrz3kpnDWJuepHLFFasg8G</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>o5tBXm4fwqfqMPM3vCqSBh</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>dasej87500@1200b.com</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Yy8oXIO1WwhAs52GIyfz8cvB61j5nEn0</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>BdQLNFvBk8rXam7mrfrSvi</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>hopib72551@coswz.com</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>MeX6ONhKqkQ9OqJ1B2Fqe3Sk1jDxhYid</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>ecHttQ5Codf5ui92vMCuCB</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>jelib91917@1200b.com</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>izQNb2AvCgWrplowzT1kkmuwtsk9uXYS</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>iZwmPXRfHddnLmMk2949sD</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>mitopar920@coswz.com</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>1BQOnHrryDP8g0f8rEghxfIhrmYHAUfz</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Y6sSECZLxeaVAVixgLPD7j</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>nipibod949@coswz.com</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>8cyOycwNqr8j3NhYOcYra1b8jZ7inrol</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>2GzA7SqvnWFviQXgAoTvnV</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>himin58719@1200b.com</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>SWnYpCh6288IUlI2fuZceQU2W9JfjQST</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>H7bsBfYQ8BrVwWrPHqLjcN</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>pikowij645@coswz.com</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>qSovfnE9o9mF3ImMFf4rs1ekuQzLAb3E</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>nsNw9zroEK5eFFqvCXnWdi</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>kimocas384@1200b.com</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>ndaZlzoJCEAL2rWcFOEeuMKSrrA132tV</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>QM6aymxo9BHCksxvTUwwSp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>himir10395@1200b.com</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>CQij8YQXSpkKVOXeFtwUVODsQsA7a90U</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>c7cz8t6G2RZKScjBvfUg7C</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>xepare8732@1200b.com</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>3QDOjoOra9UuXpWy9msW49rTC5ST62np</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>aXex4ccbsE2NoxKU98uJcA</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>nikeyem927@coswz.com</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>xgVqH1xBNsc07baDwB7HbSI9oXDZ4Mbe</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>9oXLgTF3t5eZipeHdDxkoN</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>carom36612@coswz.com</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>FYj1dKSpiJ8Ut1ZBkYbRmXo1pMMuxqHD</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>wCdZzBTZ7ZuodXp9VGrQ49</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>jefico4433@1200b.com</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Mqronv3aPXXeVMU7h4rEQ98jYqdM5Qj9</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>EniW9QPTGrEsgZjG6LsZvh</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>refok65788@1200b.com</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>HQm2YrQjWztQPeS5tcn9glppcbhJgFSt</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>pLgwMcrhZTMpJJhJcvTsMk</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>jifol26170@1200b.com</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>g94mApVW76Rn8IyAUSEVwQGPPdlzJ716</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>CicMLCpuGezkjGk5BRuPtN</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>benefi4649@1200b.com</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>GKS85X1OyHVpcXEJuYyprwl1cdFr6kF2</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>9UhfydYnajbpbavk8CffTd</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>sopike5287@1200b.com</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>mPbhTO5MojzLRb1C68gnFHwzwX7ItMw4</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Xkha5cEeszxEHfushaQdw4</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>karec14107@coswz.com</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Pev0PSY2mI6oAqhMLWS1CqkYNrw5fE8d</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>EAinmt9dJmQMnyqKX7WWbE</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>xavopo3145@1200b.com</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>haMuanIGVhHXeJ2MsGI7M12LJ6ZZXsaT</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>AQiQV2BBAz6jwafepoNqbf</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>joriwex207@coswz.com</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>kHUOAfblQhaESv3Jjp0IbNlEaussgW39</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>V2csbEQ9pMFz4QUJg2jJ6i</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>voyafo9058@coswz.com</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>FpOlWZ7m2j7npHqz1ZkT3FJ6dF0cLSxJ</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>2W2tMtPupoVuhB3oHRLJp9</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>lexano5101@1200b.com</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>6nB2pRvb5tqXvU0CrEJx5wl3nUhgIuRv</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>ZVYAVAPRaaXmrdPRb7ZELh</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>kirotit859@1200b.com</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>8m6mEMsePqy6GXE49ruSBO8u1f9s0qNi</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Rb4nWVdb23evtoAQ8JrG8T</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>navet16470@1200b.com</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>BMo85M8uWXIKo419Gh45BgP3QEkWemSv</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>beStJTkVbLtQPnJEeEHkjG</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>sodeh73836@coswz.com</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>PsVbxG4qvaLmmT8wqHmHpIqdWmCQ5d3C</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>K6kEmvdTNsZnJBjHhMSvbP</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>lovofes117@1200b.com</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>cZgYvZLIybqw9ARhD4QkpometnbkysUv</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>GMMBiZmGifzYF28fSNa9c2</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>pamopi3411@1200b.com</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>PkRugnvBD3B0igMREwLPLg3sl9oeM90B</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>UCAPmEkfidSk7cYerjyxdd</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>jifemo1970@1200b.com</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>imFLpCaYo6XcRqSJPCZfL11ncutZMANJ</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>YrCYE3si4V7NcbWqAVMGCU</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>delorow382@coswz.com</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>ukwJiuR0KTAlWweTSyXXnBtkyyta26Ux</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>BN9GkFz8CciG6LUKmXDXua</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>podor68087@1200b.com</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>vgsDZN5NG4tWhlactb1QcYZMGtdRQHbZ</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>8x4oUL8G2mR6HBJFVj4XAc</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>wayawa6952@coswz.com</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>oIeAeQ2KtbS65uf3b2UisJvaxPsFfi6Q</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>bpeArChpJhbFCVnmZA8RJ4</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>firav95941@1200b.com</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>EqocVcwKEhjCDmFVeP8tFBRJ6IEZw9Hd</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>VqtQ6FHCbuaGK3kZ2evggF</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>todel27954@1200b.com</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>xCOoFb986TXsBpIdSftqiOtUC4cGb47c</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Fmt2DRp7qgWkbYW2cc5cBT</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>cemide9890@1200b.com</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>xz1XAl9C6EBI0Orzw4N6MxLU4vefQ8gu</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>8tm9YXNQzyNeLuUwYUJUXG</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>bohicol233@coswz.com</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>HEIaGbLUQZL3aBgiU7DeODVxM5mzztv9</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>kc7BafimJ7mQZpmfam7b8J</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>felabar963@1200b.com</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>nrzMpcvs2P0JgXR56hQdwYuf4OVcAcoz</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>9qcuYZqxJYHguQn6aAFc8P</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>ritam21886@coswz.com</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>oxiBCBlg1ptibwUlGEY5t4WOGUpGuJjY</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>sGDP7kcxiChZc2Bx4sLPeF</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>lolama3392@coswz.com</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>EYStM48As8IXr1nfwIM4WxZ1qJUTJX2e</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>ZR4i66bB2VXLrodxE99pUQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>yevac45467@coswz.com</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>sfuWuiw2opt5IFJZ9UMJDLGqieQsLduG</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>xkhpQ7axLsvj9WvL2eQUxW</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>wekake2133@1200b.com</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>F9H7VSAxhKrx5C25wW4mtgjCHy80HG68</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>tzsMtZDzfe7SiYigYvy2Lc</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>vejeme4671@coswz.com</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>yXXEkV1j5kwyJLZMLNiQsByYIPZ04OlS</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Z28jCiYicjtyokHCZWJrEB</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>sivoman409@1200b.com</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>UvuMKxJ5htjJs1ok5OpPyll5RfEPiF8I</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>5FguZ3Zn6C3aB8LniffP3J</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>tejeme6947@1200b.com</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>9NRHZ5QTuYdkqyzDB4WGQFDbb9cKLdQX</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>SqFCfMEzZTi4KWbuHhezve</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>yaxibos654@coswz.com</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>YojEjoF9kICucGwWEfRkwQ3jXntmXUb9</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>qJc3QqXhppN7f5csRN7CJk</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>kosiled837@1200b.com</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>G5PjiRNVix9C8vDatmUm41lbkBl7zADA</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>DrdxVJAQGaCp3rH5MPcjCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>bejecim416@coswz.com</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>ZK8oqUNYpic5xam0Dw3AY32KRu0YheUA</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>uapU7itjAMBfJZqzh6JSoR</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>noyawer694@coswz.com</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>LizuAtiXfe3CL8Trx5TvTHn4Kes47XMh</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>9iNybNN6AYXRphPZBfiYu3</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>rawapel384@coswz.com</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>YaDZvBU1AnaZj5jASC649lSTNWyx5MEd</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>VH4wL9DJn7CJeVLxiNrsPR</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>milori7781@coswz.com</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>hFzcNXFLoAqcdPGmun9l7WEFqpAmEOaS</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>DzVhcmiQoCj9GNGyEey8bV</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>xaget22612@1200b.com</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>fQVioJODzFUzLVYuLuIh4GMtytZflRa2</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>hkoGzZKufWxrN2Veqi8KRF</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>lafan29114@1200b.com</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>YFxXU1c8VvbfKyipOr8bD0YShmN7DEvR</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>aiRF35cN6FcH79ipXTRLXf</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>rokiji6230@1200b.com</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>ygvcE5DYxeHUxkG0wLgqMpGu5T5EEUlr</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>djbf85rvyrKiLwcLZKQWJB</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>gajaxev858@1200b.com</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>PzeCOI1TNljRaIjGXQ9LB6umxkv7CkXi</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>4hTFeDdCkMpPpSwi5ZQdGD</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>wakoxah547@coswz.com</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>XndyveOS7Kzyh7lKdJBfPE2uG8YRCMEB</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>5pJUDPketCPoLn9bg8Uw8a</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>hekesip792@coswz.com</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>IddzLbWJBLCstiPwMcSKtPUGIRAJes7I</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>bE9WSksfdHYTuL7sctbf9E</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>desit76037@coswz.com</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>GdRWQWMORdsVhopWYKd0vkgyXhFjnEEm</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>uSiJ39RLf2ik3RcUnewL78</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>hokilo8846@coswz.com</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>xy3p1a3uJzHXNrTKPBgOo8gcByWlQVbf</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>SkV6iQWbr3uX4qAxZMqJ8e</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>kinota3968@1200b.com</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>tVo6QytEZJhSedhbNCxuNlr6TtbDTwbG</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>GBi9PFWwb6jZvBR6tHt6tG</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>kafok91274@1200b.com</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>rbSl44jvfMA0O1AgoBGn8yotnX4At9qj</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>P8CJeHZPafJ9ksK4DjP9X4</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>hepivov461@coswz.com</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>LRWAtBvcP3OHzMNpy4pAmYoAZKt2Hzd7</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Wq2676chbay4PApch66btW</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>mediga6962@1200b.com</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>f5v44bGLXo945pbByUKgRRBtJrOLwV9s</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>2pf6YtJVvCcCQ73GoeTwkG</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>gemesiy261@1200b.com</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>43dDJwRPPcXgqxtpic1C8qgV5FnwTjoN</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>DfBW3WCK6YBxpRNpfYyFsS</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>vopop36078@coswz.com</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>ihYvMGMIiZdbtiNoT3cuAQVhOy7oai63</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>JipTjAkfWuMRyWMsSHXbRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>liviyi2687@1200b.com</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>5O8UznvS5fiwcl2Iqg0EU6LvuZfsalGa</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>c6MJ9qBahPoXcZnmu3LTad</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>nojivi9674@1200b.com</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>2RhHD9yV3vccBEgtzrMnZ8Rq4HTzeh8W</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>ZcBcVFnKUGXyRi8xZwzpCC</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>fixeti9021@1200b.com</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>d7L3aNaXEKjfO4tFSBNkUVJbD8ZLNnSJ</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>qqJBK3ioMf58qe4eaurhiM</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>widas71479@1200b.com</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>55QYbQFAmv3hQrOaVpTXtNmpsU1k3dPO</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>KVtEYD5bCvywZq65oaCDnb</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>bawavip104@coswz.com</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>JtZpye7pdPl6lK7UTCMhuZoY2hvyJ9pK</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>mTJtCxtdppM3YpyJcQDFkS</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>copawo7293@coswz.com</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>B0Mc8vRk33LEEYPIhYNJ6GOBTsBtC7Kx</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>yNVgoudEmCGXPJy5TKYFuJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>yociko1703@1200b.com</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Uu7qo08f3qrpYeZGiovbd4b6fMvJpg5T</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>w4bB4KNZafhZtw8Dv7Vq7c</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>yohiho1186@1200b.com</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>y1ROvKdGD3IfK2LpQJ6emLeiryUyeTOy</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>U3eNhDLmBZ9kbbgQuTJggg</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>vepek51758@coswz.com</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Xd0XnvFWpuYJb6EyX4v0qZGJyzKPbpjf</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>K7wD42ADsf3yKih2DpdZX3</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>vicexa9591@coswz.com</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>npz20JjzNH92wIH4tCQx49nC0it14Xxw</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>rZd7CALt2MZEMHmpDtGQxB</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>hecab14854@1200b.com</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>K8wwgIDz5G56KxRoP7JgMK2PO7C2UzvN</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>4KT5DztHkEUnCgYrNhRx4e</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>carexan555@coswz.com</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>cBLSH97sWXVnfO4kUKBNbM8eYNZcanHx</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>HW37WS2fucmm8m6ZUSMU7Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>lokos77574@coswz.com</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>rNU7s0xkwJcc3DDFI9osfwRqVJB5MUvd</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>777awg7nDxL7oVL4duMc6h</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>nojex76241@1200b.com</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Kz7OdwkMZTZaDJQ1iUTZLbGvoS84keOP</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>hVpkXzmpNbzDE5fFtiJbc2</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>hovifim988@1200b.com</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>CK0Wp6WKiFD7acjl10G8vysxWR48wZRg</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>P5XJ2dTaNUHsMkCoMgVS8i</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>yawoc12567@coswz.com</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>uT6UL7Qo9WWZFIw6nFihvEoPsRuWB2cB</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>J8JUeTV2yxn9wmuA5vLnfW</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>gecadac197@coswz.com</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Grzwxyx41AkWP5m4f3xtEu0JlfrFim7P</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>SARbUSMkNZD9XjpwUeK4oH</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>goyixov775@1200b.com</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>h6VvXzCUwwTE11bRqNCZS8brKBY5zCbz</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>REZRkCf7tSD37FJmyWRET3</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
           <t>jayit97735@1200b.com</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B162" t="inlineStr">
         <is>
           <t>xstn0Y1QeBj5bnDGrXeOn648TCmCcc0G</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C162" t="inlineStr">
         <is>
           <t>9LJtRkXV4MTjAwMVwgoUaf</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>tiyeciy866@1200b.com</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>3P4jyDaUqq5fdNqWDIb34rlZbRf2KCxG</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>RSr7tgrfTd94Mm3owU2Ry3</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>racek36029@1200b.com</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>hDghGPPIJ1UDWE5TaZJEOsOhg3DQYHkJ</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>V3rPPRdJNBBWxdp37MKNZg</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>lenac61027@coswz.com</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>xCgpDNXZ0OxWUZTv3cCs15Fx5gcmbGih</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>JrV6Aq9rfLw9W5Kf8jPry4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update auphonic processing logic and add auphonic_standalone.py
</commit_message>
<xml_diff>
--- a/settings.xlsx
+++ b/settings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C165"/>
+  <dimension ref="A1:C164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,2752 +470,2735 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>sekeber866@dropeso.com</t>
+          <t>fatisis252@filipx.com</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>6m6Boofi3vyiye1mWGk2z8JPLedRYP1l</t>
+          <t>xXM7YgF9EfC9ObxBpbjd3oUxmIDj0E1J</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>mqhhwkNjs6LbnusE87WgxF</t>
+          <t>H9k4tH57H8Qx2xxkDgw6ZJ</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>fatisis252@filipx.com</t>
+          <t>xaxaveb930@gamepec.com</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>xXM7YgF9EfC9ObxBpbjd3oUxmIDj0E1J</t>
+          <t>Lm3LOfqVcTHWIgPEXPokowvo21CayIGZ</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>H9k4tH57H8Qx2xxkDgw6ZJ</t>
+          <t>oJkWc6d7ikC8p8z5VRMZii</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>xaxaveb930@gamepec.com</t>
+          <t>socamog235@gamepec.com</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Lm3LOfqVcTHWIgPEXPokowvo21CayIGZ</t>
+          <t>80M9YjLNMMpnHxvn77VqlwjOoygXqTJJ</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>oJkWc6d7ikC8p8z5VRMZii</t>
+          <t>mxPwz4s5mtD9TAxE6AkNeb</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>socamog235@gamepec.com</t>
+          <t>rerob43025@gamepec.com</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>80M9YjLNMMpnHxvn77VqlwjOoygXqTJJ</t>
+          <t>GWODyKNPNpFbbugHbLAexY9EO4QfQgPN</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>mxPwz4s5mtD9TAxE6AkNeb</t>
+          <t>uKzUdj8mUViiqMpRne6qse</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>rerob43025@gamepec.com</t>
+          <t>wonagay313@httpsu.com</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>GWODyKNPNpFbbugHbLAexY9EO4QfQgPN</t>
+          <t>JvazbN1rE4hVvXvj8QcyNGzf9sg5Xmxk</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>uKzUdj8mUViiqMpRne6qse</t>
+          <t>9Tkxna4xBVXypXC4Z9TdHB</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>wonagay313@httpsu.com</t>
+          <t>figalab281@idwager.com</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>JvazbN1rE4hVvXvj8QcyNGzf9sg5Xmxk</t>
+          <t>Xw4UIPg7EoCNOkbQF4LFxF1ixbErLtBU</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9Tkxna4xBVXypXC4Z9TdHB</t>
+          <t>jvMnLJVUmZrnt6uGnpArES</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>figalab281@idwager.com</t>
+          <t>rinepo9302@idwager.com</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Xw4UIPg7EoCNOkbQF4LFxF1ixbErLtBU</t>
+          <t>sE3j0F88W18qS6xZegJpw9dYUlLOQwF8</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>jvMnLJVUmZrnt6uGnpArES</t>
+          <t>HXjPdNqjJZbmLYnUajk8Nf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>rinepo9302@idwager.com</t>
+          <t>hoboxo4549@httpsu.com</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>sE3j0F88W18qS6xZegJpw9dYUlLOQwF8</t>
+          <t>OuWxiJIp9xmP2fopYIDPJgXuV6gC7g5R</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>HXjPdNqjJZbmLYnUajk8Nf</t>
+          <t xml:space="preserve"> y4BhwAH4FDg4cC8QQHDVKB</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>hoboxo4549@httpsu.com</t>
+          <t>xefes61540@httpsu.com</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>OuWxiJIp9xmP2fopYIDPJgXuV6gC7g5R</t>
+          <t>1YEdnC1nUvGW7P1hEGehAs8os2fzoEhp</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> y4BhwAH4FDg4cC8QQHDVKB</t>
+          <t>n38HSjtVqUzK4bLNXgg9wA</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>xefes61540@httpsu.com</t>
+          <t>dipah74837@httpsu.com</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1YEdnC1nUvGW7P1hEGehAs8os2fzoEhp</t>
+          <t>NlidtI9aaO82ajLNo7AryVWkMNYeItXd</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>n38HSjtVqUzK4bLNXgg9wA</t>
+          <t>ZTXVi2xiJJzSLNRe4yxeX2</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>dipah74837@httpsu.com</t>
+          <t>nawat37231@roastic.com</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>NlidtI9aaO82ajLNo7AryVWkMNYeItXd</t>
+          <t>FdXCpc87a5uQhVaqntEyZzjryF5rlACw</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ZTXVi2xiJJzSLNRe4yxeX2</t>
+          <t>ycGayRsKw7WvUeSsMdjz5Q</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>nawat37231@roastic.com</t>
+          <t>varaf33883@naqulu.com</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>FdXCpc87a5uQhVaqntEyZzjryF5rlACw</t>
+          <t>531lLSFzKRS2pMW7R6AjQyoYg0nJfSfQ</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ycGayRsKw7WvUeSsMdjz5Q</t>
+          <t>i7H4EWbcteZc93wmisovt4</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>varaf33883@naqulu.com</t>
+          <t>fetip10878@roastic.com</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>531lLSFzKRS2pMW7R6AjQyoYg0nJfSfQ</t>
+          <t>7SZJWYq9ZbsEnQiZ7J2NapfHWz6q5z39</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>i7H4EWbcteZc93wmisovt4</t>
+          <t>bJCYMBgi9ifri7qi8HFWy3</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>fetip10878@roastic.com</t>
+          <t>hexori1127@roastic.com</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>7SZJWYq9ZbsEnQiZ7J2NapfHWz6q5z39</t>
+          <t>oNV0c2SijXp7CxRlzuqivcRZ3wo5VZBf</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>bJCYMBgi9ifri7qi8HFWy3</t>
+          <t>wyW6Rqxu8K8TYkgVPsKeKn</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>hexori1127@roastic.com</t>
+          <t>linide1021@roastic.com</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>oNV0c2SijXp7CxRlzuqivcRZ3wo5VZBf</t>
+          <t>ZeVGmMKpmGC4OZjycckcVFyijfXwHksS</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>wyW6Rqxu8K8TYkgVPsKeKn</t>
+          <t>2oPnuNvyrRsUbQMuRq9oVA</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>linide1021@roastic.com</t>
+          <t>licav42884@naqulu.com</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ZeVGmMKpmGC4OZjycckcVFyijfXwHksS</t>
+          <t>hnL1dYZNWM8b8MEWTHA6CKsNWjvxkT5D</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2oPnuNvyrRsUbQMuRq9oVA</t>
+          <t>vm8ggtLTbzzcBRMr3MGRVc</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>licav42884@naqulu.com</t>
+          <t>gopev53591@okcdeals.com</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>hnL1dYZNWM8b8MEWTHA6CKsNWjvxkT5D</t>
+          <t>I0Z17qFrx7c995zbgVrqLtMM0Y6dd3h9</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>vm8ggtLTbzzcBRMr3MGRVc</t>
+          <t>JgjHU3eCEeDCuM2B86evam</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>gopev53591@okcdeals.com</t>
+          <t>dohojev953@nctime.com</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>I0Z17qFrx7c995zbgVrqLtMM0Y6dd3h9</t>
+          <t>7C3qfKLEE02rUw9YCXynmrGxNPCdtKuc</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>JgjHU3eCEeDCuM2B86evam</t>
+          <t>HMq3qgxGHux8TjvJGPRKMg</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>dohojev953@nctime.com</t>
+          <t>yamocot925@nctime.com</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>7C3qfKLEE02rUw9YCXynmrGxNPCdtKuc</t>
+          <t>wht7NqRuiTvgrqaJpsxTVXxyXRnPRLDu</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>HMq3qgxGHux8TjvJGPRKMg</t>
+          <t>rrXyG64aA6K434NmqnBkok</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>yamocot925@nctime.com</t>
+          <t>widivav664@nctime.com</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>wht7NqRuiTvgrqaJpsxTVXxyXRnPRLDu</t>
+          <t>myAJcAFPf3e7OE0ESDmS5qqHoEpqPhda</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>rrXyG64aA6K434NmqnBkok</t>
+          <t>fhAoCcEiijeJi3rtgDuNNd</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>widivav664@nctime.com</t>
+          <t>gebasi3686@nctime.com</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>myAJcAFPf3e7OE0ESDmS5qqHoEpqPhda</t>
+          <t>RB9t58YEm0itLBhHXspWtsx9qsB6DB9e</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>fhAoCcEiijeJi3rtgDuNNd</t>
+          <t>Re4Gua6CJgPQvGKHyWtbFn</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>gebasi3686@nctime.com</t>
+          <t>racirop308@roratu.com</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>RB9t58YEm0itLBhHXspWtsx9qsB6DB9e</t>
+          <t>Fp9aCSPL3V5biVE0mZDCJJHY6GDBDILv</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Re4Gua6CJgPQvGKHyWtbFn</t>
+          <t>FnytnEAHavuLvStPGYoMAg</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>racirop308@roratu.com</t>
+          <t>kilov89341@nctime.com</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Fp9aCSPL3V5biVE0mZDCJJHY6GDBDILv</t>
+          <t>Sr9kw7c7zNpGtvhRS0MLO9H8npfMegLZ</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>FnytnEAHavuLvStPGYoMAg</t>
+          <t>4dYrE6SS5dSxt5qwTvzTVT</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>kilov89341@nctime.com</t>
+          <t>gevel44383@nctime.com</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Sr9kw7c7zNpGtvhRS0MLO9H8npfMegLZ</t>
+          <t>bwyzzEVRYYttA7tmYbgsy4xcw7UVgV8O</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>4dYrE6SS5dSxt5qwTvzTVT</t>
+          <t>HzPXvuSXXQ6S7iCQmMeF9T</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>gevel44383@nctime.com</t>
+          <t>fixes12536@nctime.com</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>bwyzzEVRYYttA7tmYbgsy4xcw7UVgV8O</t>
+          <t>tLFSJBbymOOz3JjD6B8Za7wIo9b5reiE</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>HzPXvuSXXQ6S7iCQmMeF9T</t>
+          <t>xuqgf72emBu6atQU9KJPwC</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>fixes12536@nctime.com</t>
+          <t>goyima8506@nctime.com</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>tLFSJBbymOOz3JjD6B8Za7wIo9b5reiE</t>
+          <t>g7H4uFMeYmfFQlN0y5i2GvHrqHojlJ1n</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>xuqgf72emBu6atQU9KJPwC</t>
+          <t>gXDsBP9zWswMC32WWBWfAj</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>goyima8506@nctime.com</t>
+          <t>nekidi7850@roratu.com</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>g7H4uFMeYmfFQlN0y5i2GvHrqHojlJ1n</t>
+          <t>MC0690dIR7s41wFmAsVT84JN5gGRF4Q8</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>gXDsBP9zWswMC32WWBWfAj</t>
+          <t>zrV8izMTZxKtZeUdkketVA</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>nekidi7850@roratu.com</t>
+          <t>wofetef124@jparksky.com</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MC0690dIR7s41wFmAsVT84JN5gGRF4Q8</t>
+          <t>bNv5oiinBiebNL2MPIq8hGZx3CXVH0jm</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>zrV8izMTZxKtZeUdkketVA</t>
+          <t>hPBtQoQTuyiDLzW27UVAbE</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>wofetef124@jparksky.com</t>
+          <t>daseso2631@jparksky.com</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>bNv5oiinBiebNL2MPIq8hGZx3CXVH0jm</t>
+          <t>DRXjVQctFOWz1cQcUQODfryiXg31FjiL</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>hPBtQoQTuyiDLzW27UVAbE</t>
+          <t>MtHkkP5Qk2RR9zVA5gLgy9</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>daseso2631@jparksky.com</t>
+          <t>ririwa4119@ixospace.com</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>DRXjVQctFOWz1cQcUQODfryiXg31FjiL</t>
+          <t>mcByeqm6xZDW1STLVQ8tmtMWVD4OZ0vq</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MtHkkP5Qk2RR9zVA5gLgy9</t>
+          <t>NkaahaDx6Umohs8fhs3x7d</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ririwa4119@ixospace.com</t>
+          <t>neloc13413@akixpres.com</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>mcByeqm6xZDW1STLVQ8tmtMWVD4OZ0vq</t>
+          <t>5tn4iP1EdUCal3f7dlInF9hcZRWoDDam</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>NkaahaDx6Umohs8fhs3x7d</t>
+          <t>dHpjvBPUa5g8Ka5MQu8A34</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>neloc13413@akixpres.com</t>
+          <t>cadol56750@atinjo.com</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>5tn4iP1EdUCal3f7dlInF9hcZRWoDDam</t>
+          <t>JAvZf5v9odlVKpCQm04PEJIp9Qlma8be</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>dHpjvBPUa5g8Ka5MQu8A34</t>
+          <t>Dw7R7kP9dU9R5dw2ACuYee</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>cadol56750@atinjo.com</t>
+          <t>gigij73348@akixpres.com</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>JAvZf5v9odlVKpCQm04PEJIp9Qlma8be</t>
+          <t>6uBAE8WK2oNHLqUP1scuIX5dvPgqkk6W</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Dw7R7kP9dU9R5dw2ACuYee</t>
+          <t>XiYeYgHxXcnH2tbqEBxtnk</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>gigij73348@akixpres.com</t>
+          <t>hipota9018@atinjo.com</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>6uBAE8WK2oNHLqUP1scuIX5dvPgqkk6W</t>
+          <t>LxXoRVMl9zQRFnQ28SrktX3U2GyHcOOh</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>XiYeYgHxXcnH2tbqEBxtnk</t>
+          <t>Fx7zZF5qibuBBHkUGq6xpC</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>hipota9018@atinjo.com</t>
+          <t>gigemi1270@atinjo.com</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>LxXoRVMl9zQRFnQ28SrktX3U2GyHcOOh</t>
+          <t>rsmqBLdT1vuYrCZ9rNoOuXVzZHSi6IVL</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Fx7zZF5qibuBBHkUGq6xpC</t>
+          <t>WKZzU8yHMSTUMeJKtNCB9W</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>gigemi1270@atinjo.com</t>
+          <t>veyorox418@akixpres.com</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>rsmqBLdT1vuYrCZ9rNoOuXVzZHSi6IVL</t>
+          <t>elL3annwEMcNszO8xI31nd9akdmbMfut</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>WKZzU8yHMSTUMeJKtNCB9W</t>
+          <t>bJxx8YodEXUUTKXaNmTN3Y</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>veyorox418@akixpres.com</t>
+          <t>wahesen320@atinjo.com</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>elL3annwEMcNszO8xI31nd9akdmbMfut</t>
+          <t>Q15kREigAFjMZLUAyW1QftIpkSUpm3Zx</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>bJxx8YodEXUUTKXaNmTN3Y</t>
+          <t>Zs9EHCcnZyWv3X6iCBbiaQ</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>wahesen320@atinjo.com</t>
+          <t>bagabe8853@atinjo.com</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Q15kREigAFjMZLUAyW1QftIpkSUpm3Zx</t>
+          <t>0bAH8FOjsLlu1jeIoirXHcN3hmXZ9Ll7</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Zs9EHCcnZyWv3X6iCBbiaQ</t>
+          <t>m9uGnynHJsabaD2Pyzyenn</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>bagabe8853@atinjo.com</t>
+          <t>riwag56154@akixpres.com</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>0bAH8FOjsLlu1jeIoirXHcN3hmXZ9Ll7</t>
+          <t>SnxsC4IIztaAh8Qk0WXFN6qDc4WFf9DO</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>m9uGnynHJsabaD2Pyzyenn</t>
+          <t>Qv3KsYMDxnp7thHQHZNfPS</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>riwag56154@akixpres.com</t>
+          <t>wepol47565@akixpres.com</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SnxsC4IIztaAh8Qk0WXFN6qDc4WFf9DO</t>
+          <t>qw1WKJ4bDDImTMqzZi9eXLwHHkQpTSO6</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Qv3KsYMDxnp7thHQHZNfPS</t>
+          <t>CxXPjugqjFd6CAAuf8HZaV</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>wepol47565@akixpres.com</t>
+          <t>solego9606@atinjo.com</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>qw1WKJ4bDDImTMqzZi9eXLwHHkQpTSO6</t>
+          <t>9gDLSKh98F9c2SSUvuJSAr6MszvcTTLi</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>CxXPjugqjFd6CAAuf8HZaV</t>
+          <t>NrJch3iCXMJM9JLFxymFtg</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>solego9606@atinjo.com</t>
+          <t>wafile9558@akixpres.com</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>9gDLSKh98F9c2SSUvuJSAr6MszvcTTLi</t>
+          <t>8tjVlDYXKoiKA9LiMXOL0Pjypq1xvhiY</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>NrJch3iCXMJM9JLFxymFtg</t>
+          <t>wYwfXdMpdgViJvhHhNePnd</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>wafile9558@akixpres.com</t>
+          <t>ratad81098@atinjo.com</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>8tjVlDYXKoiKA9LiMXOL0Pjypq1xvhiY</t>
+          <t>0YdxGb2ITKezrGWiFa9cn7k4jOpQgO8c</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>wYwfXdMpdgViJvhHhNePnd</t>
+          <t>myUuzuxSbiP7xdYD6mSd4K</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ratad81098@atinjo.com</t>
+          <t>yataven591@atinjo.com</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>0YdxGb2ITKezrGWiFa9cn7k4jOpQgO8c</t>
+          <t>ozoo16Bl6Q3dPwhmbTdvYncz362cRwXP</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>myUuzuxSbiP7xdYD6mSd4K</t>
+          <t>RuVixv8g3X98fMcL9cDqRV</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>yataven591@atinjo.com</t>
+          <t>noder31454@akixpres.com</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ozoo16Bl6Q3dPwhmbTdvYncz362cRwXP</t>
+          <t>5wR46xR4wULRGza81qbyC3Dux2fCm4RK</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>RuVixv8g3X98fMcL9cDqRV</t>
+          <t>yrnwYNcvGrUNj4rKmm2svH</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>noder31454@akixpres.com</t>
+          <t>boleg64834@atinjo.com</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>5wR46xR4wULRGza81qbyC3Dux2fCm4RK</t>
+          <t>WfrxUSz3OnBtuoVSpin6wSQbymWavST2</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>yrnwYNcvGrUNj4rKmm2svH</t>
+          <t>DuwptNFqTjaNPX9dH7ban7</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>boleg64834@atinjo.com</t>
+          <t>kisagiw989@akixpres.com</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>WfrxUSz3OnBtuoVSpin6wSQbymWavST2</t>
+          <t>xM16sQ7DLf5h2ELiGcc5ZeEeZr7G5liw</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>DuwptNFqTjaNPX9dH7ban7</t>
+          <t>MY5dmNN2Wj95atQyKcRWtD</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>kisagiw989@akixpres.com</t>
+          <t>jehego4595@atinjo.com</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>xM16sQ7DLf5h2ELiGcc5ZeEeZr7G5liw</t>
+          <t>nFC0pqugt0SvyHWfFImqKozyvuIASodz</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>MY5dmNN2Wj95atQyKcRWtD</t>
+          <t>eoxChE5ZREvYNCZkZr2xF5</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>jehego4595@atinjo.com</t>
+          <t>dexexed273@atinjo.com</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>nFC0pqugt0SvyHWfFImqKozyvuIASodz</t>
+          <t>4sEBwF29AkejGdLQ7cNm4V46UrtlZL51</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>eoxChE5ZREvYNCZkZr2xF5</t>
+          <t>tqS5U8xzqPKuDatqWxTDAe</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>dexexed273@atinjo.com</t>
+          <t>reloriv513@akixpres.com</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>4sEBwF29AkejGdLQ7cNm4V46UrtlZL51</t>
+          <t>0BAbfCRMLqLnNR0SGk1zdCfIDpU68ozw</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>tqS5U8xzqPKuDatqWxTDAe</t>
+          <t>8ziLdQSvxoHJFBm7bqx8gK</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>reloriv513@akixpres.com</t>
+          <t>lejepas261@akixpres.com</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>0BAbfCRMLqLnNR0SGk1zdCfIDpU68ozw</t>
+          <t>1H9QUd3bfLCMmPXprcuq6oA6P0cZZuOi</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>8ziLdQSvxoHJFBm7bqx8gK</t>
+          <t>FrF9e7kRqvwzk8QZzucCrB</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>lejepas261@akixpres.com</t>
+          <t>jegosi2800@atinjo.com</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>1H9QUd3bfLCMmPXprcuq6oA6P0cZZuOi</t>
+          <t>pRQrdbkcm8eTsnecHWkvzCDhcxlN0zgo</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>FrF9e7kRqvwzk8QZzucCrB</t>
+          <t>RYdSN2H3oa9uobCLnUWGrN</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>jegosi2800@atinjo.com</t>
+          <t>naxelaf699@akixpres.com</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>pRQrdbkcm8eTsnecHWkvzCDhcxlN0zgo</t>
+          <t>HLhpdosj0jR6TKxbcXXsZyesgfGf1AUt</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>RYdSN2H3oa9uobCLnUWGrN</t>
+          <t>gUM4qvu9Yvo94aDx7ZsyS6</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>naxelaf699@akixpres.com</t>
+          <t>yewewod514@akixpres.com</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>HLhpdosj0jR6TKxbcXXsZyesgfGf1AUt</t>
+          <t>HsP1XnIRh2vmG847Ps4LhmL2XHHMtuf8</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>gUM4qvu9Yvo94aDx7ZsyS6</t>
+          <t>JATjdyhEfXsitwrsdw4UaP</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>yewewod514@akixpres.com</t>
+          <t>secotot918@akixpres.com</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>HsP1XnIRh2vmG847Ps4LhmL2XHHMtuf8</t>
+          <t>6wHZfUI3LUTYbuTpmKSvHdtVj3zTsU6E</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>JATjdyhEfXsitwrsdw4UaP</t>
+          <t>kS8op9jKuQk6RS8wHZGDUR</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>secotot918@akixpres.com</t>
+          <t>micis44451@atinjo.com</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>6wHZfUI3LUTYbuTpmKSvHdtVj3zTsU6E</t>
+          <t>fDRR3GWUvhnQQxW0yZSu2xwBMggGBylV</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>kS8op9jKuQk6RS8wHZGDUR</t>
+          <t>yMJ57L5SAmDiAFHoMv2wUB</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>micis44451@atinjo.com</t>
+          <t>banode7154@daikoa.com</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>fDRR3GWUvhnQQxW0yZSu2xwBMggGBylV</t>
+          <t>JCOSpFLRw8eGUdGUPalob9DnXs14cDFu</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>yMJ57L5SAmDiAFHoMv2wUB</t>
+          <t>CYzAi4iqRtq9Lp8iYQVYDG</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>banode7154@daikoa.com</t>
+          <t>yelar54822@daikoa.com</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>JCOSpFLRw8eGUdGUPalob9DnXs14cDFu</t>
+          <t>s6JOCcXKLapyRPCZ0K7kcCTu8zRVIh6P</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>CYzAi4iqRtq9Lp8iYQVYDG</t>
+          <t>s4KF4kgtwvwqzNAETSBkEn</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>yelar54822@daikoa.com</t>
+          <t>gibino1422@dretnar.com</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>s6JOCcXKLapyRPCZ0K7kcCTu8zRVIh6P</t>
+          <t>nxTKC2GLECZuRdJqNxWu4FueMG6FCSss</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>s4KF4kgtwvwqzNAETSBkEn</t>
+          <t>wFCv2kwYEyRRBTQRWZDmWG</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>gibino1422@dretnar.com</t>
+          <t>tinowa6684@dretnar.com</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>nxTKC2GLECZuRdJqNxWu4FueMG6FCSss</t>
+          <t>u5QKv1tzXgAuwkwmGeUdosXqJf3YE0mk</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>wFCv2kwYEyRRBTQRWZDmWG</t>
+          <t>e6F7bArFz3xqHiyA48e7gm</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>tinowa6684@dretnar.com</t>
+          <t>jagala5779@daikoa.com</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>u5QKv1tzXgAuwkwmGeUdosXqJf3YE0mk</t>
+          <t>n6GPL2AghujKGoKXYFa1mDpLAN41tI8t</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>e6F7bArFz3xqHiyA48e7gm</t>
+          <t>T84oseSmPvmfZjUHVnLRtK</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>jagala5779@daikoa.com</t>
+          <t>dadac39765@daikoa.com</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>n6GPL2AghujKGoKXYFa1mDpLAN41tI8t</t>
+          <t>hldYhwMOTTzCd0VN4MiWv4PwtioXkbQD</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>T84oseSmPvmfZjUHVnLRtK</t>
+          <t>SoT9i7shyBEoBsq9pdhBFS</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>dadac39765@daikoa.com</t>
+          <t>xavimi2919@daikoa.com</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>hldYhwMOTTzCd0VN4MiWv4PwtioXkbQD</t>
+          <t>D6u5oKva8hquabzZuKEYRTRmYmn4fzlK</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>SoT9i7shyBEoBsq9pdhBFS</t>
+          <t>7TvAhBKSBeTnapk3QYeVxG</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>xavimi2919@daikoa.com</t>
+          <t>savam45676@daikoa.com</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>D6u5oKva8hquabzZuKEYRTRmYmn4fzlK</t>
+          <t>76wdvssqe4Z5TW2prOzqjNKS1X0JddFq</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>7TvAhBKSBeTnapk3QYeVxG</t>
+          <t>ermjT6fUpjdwJ8Cpbaop8R</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>savam45676@daikoa.com</t>
+          <t>wogero4961@dretnar.com</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>76wdvssqe4Z5TW2prOzqjNKS1X0JddFq</t>
+          <t>vcGKMj18D1DDq4TS3gOEF4LOLGT2x7yQ</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>ermjT6fUpjdwJ8Cpbaop8R</t>
+          <t>Bun4v3nU64AhjzpdSWiemS</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>wogero4961@dretnar.com</t>
+          <t>titow54942@dretnar.com</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>vcGKMj18D1DDq4TS3gOEF4LOLGT2x7yQ</t>
+          <t>4L16RFGlrDsOcHbpkBzt8DmJx3c20div</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Bun4v3nU64AhjzpdSWiemS</t>
+          <t>wMo7tcJSzPFdqVVwkdkhSF</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>titow54942@dretnar.com</t>
+          <t>povej18527@dretnar.com</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>4L16RFGlrDsOcHbpkBzt8DmJx3c20div</t>
+          <t>Wb2hayUo3xugCXuNWIIJdTGEsY17ZKdK</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>wMo7tcJSzPFdqVVwkdkhSF</t>
+          <t>hVxPZa2jdmwGHVj8An5hAK</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>povej18527@dretnar.com</t>
+          <t>goyaja1050@daikoa.com</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Wb2hayUo3xugCXuNWIIJdTGEsY17ZKdK</t>
+          <t>dYiibSMdcXTcy5lDePf5nXegvIAJMtUe</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>hVxPZa2jdmwGHVj8An5hAK</t>
+          <t>hqLMkRc27w7vg5CTSWwWmn</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>goyaja1050@daikoa.com</t>
+          <t>bocowa9157@daikoa.com</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>dYiibSMdcXTcy5lDePf5nXegvIAJMtUe</t>
+          <t>exrLCAXboHaXet9OlqJAN96OmKWsDnfo</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>hqLMkRc27w7vg5CTSWwWmn</t>
+          <t>hW8WWpTLfpm69rNgikkLBY</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>bocowa9157@daikoa.com</t>
+          <t>socas91504@dretnar.com</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>exrLCAXboHaXet9OlqJAN96OmKWsDnfo</t>
+          <t>zwwI8F0DewAZat1DNGEX9FDV9XrfYwfY</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>hW8WWpTLfpm69rNgikkLBY</t>
+          <t>2zQjp5rCLonb2UqmPNiwf5</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>socas91504@dretnar.com</t>
+          <t>milidij455@dretnar.com</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>zwwI8F0DewAZat1DNGEX9FDV9XrfYwfY</t>
+          <t>HfekRAMQdJuiL1IyQ2LU7Gf55ek6NEKr</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2zQjp5rCLonb2UqmPNiwf5</t>
+          <t>spQpD2WBbZirL7UNvRrpNA</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>milidij455@dretnar.com</t>
+          <t>lipota2474@1200b.com</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>HfekRAMQdJuiL1IyQ2LU7Gf55ek6NEKr</t>
+          <t>UKAWL111GeXpmJxRG6ijnrUrXau0TQWe</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>spQpD2WBbZirL7UNvRrpNA</t>
+          <t>ay2xrft7cY3VC928BPUacE</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>lipota2474@1200b.com</t>
+          <t>gidevok422@1200b.com</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>UKAWL111GeXpmJxRG6ijnrUrXau0TQWe</t>
+          <t>DtSxMlHMagZAFQHV5WiiaNI9bmqg2UkQ</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ay2xrft7cY3VC928BPUacE</t>
+          <t>NREwQMq757tnLqK3U5WoPV</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>gidevok422@1200b.com</t>
+          <t>tofepi1509@coswz.com</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>DtSxMlHMagZAFQHV5WiiaNI9bmqg2UkQ</t>
+          <t>K2qGEA8d2aRQm4p4RVVHdfWw16i1vLHb</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>NREwQMq757tnLqK3U5WoPV</t>
+          <t>7BoB84re8TsrnpfpmY5Xg7</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>tofepi1509@coswz.com</t>
+          <t>hejita4492@coswz.com</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>K2qGEA8d2aRQm4p4RVVHdfWw16i1vLHb</t>
+          <t>3lFTo0Rnbv9YiWfy3gO5xjwfHXPYNa4A</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>7BoB84re8TsrnpfpmY5Xg7</t>
+          <t>zXCFEZncTGyiQ2gaMi8fpm</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>hejita4492@coswz.com</t>
+          <t>doxixi5794@1200b.com</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>3lFTo0Rnbv9YiWfy3gO5xjwfHXPYNa4A</t>
+          <t>J6q60nEZvsFrz3kpnDWJuepHLFFasg8G</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>zXCFEZncTGyiQ2gaMi8fpm</t>
+          <t>o5tBXm4fwqfqMPM3vCqSBh</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>doxixi5794@1200b.com</t>
+          <t>dasej87500@1200b.com</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>J6q60nEZvsFrz3kpnDWJuepHLFFasg8G</t>
+          <t>Yy8oXIO1WwhAs52GIyfz8cvB61j5nEn0</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>o5tBXm4fwqfqMPM3vCqSBh</t>
+          <t>BdQLNFvBk8rXam7mrfrSvi</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>dasej87500@1200b.com</t>
+          <t>hopib72551@coswz.com</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Yy8oXIO1WwhAs52GIyfz8cvB61j5nEn0</t>
+          <t>MeX6ONhKqkQ9OqJ1B2Fqe3Sk1jDxhYid</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>BdQLNFvBk8rXam7mrfrSvi</t>
+          <t>ecHttQ5Codf5ui92vMCuCB</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>hopib72551@coswz.com</t>
+          <t>jelib91917@1200b.com</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>MeX6ONhKqkQ9OqJ1B2Fqe3Sk1jDxhYid</t>
+          <t>izQNb2AvCgWrplowzT1kkmuwtsk9uXYS</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>ecHttQ5Codf5ui92vMCuCB</t>
+          <t>iZwmPXRfHddnLmMk2949sD</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>jelib91917@1200b.com</t>
+          <t>mitopar920@coswz.com</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>izQNb2AvCgWrplowzT1kkmuwtsk9uXYS</t>
+          <t>1BQOnHrryDP8g0f8rEghxfIhrmYHAUfz</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>iZwmPXRfHddnLmMk2949sD</t>
+          <t>Y6sSECZLxeaVAVixgLPD7j</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>mitopar920@coswz.com</t>
+          <t>nipibod949@coswz.com</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>1BQOnHrryDP8g0f8rEghxfIhrmYHAUfz</t>
+          <t>8cyOycwNqr8j3NhYOcYra1b8jZ7inrol</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Y6sSECZLxeaVAVixgLPD7j</t>
+          <t>2GzA7SqvnWFviQXgAoTvnV</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>nipibod949@coswz.com</t>
+          <t>himin58719@1200b.com</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>8cyOycwNqr8j3NhYOcYra1b8jZ7inrol</t>
+          <t>SWnYpCh6288IUlI2fuZceQU2W9JfjQST</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2GzA7SqvnWFviQXgAoTvnV</t>
+          <t>H7bsBfYQ8BrVwWrPHqLjcN</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>himin58719@1200b.com</t>
+          <t>pikowij645@coswz.com</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>SWnYpCh6288IUlI2fuZceQU2W9JfjQST</t>
+          <t>qSovfnE9o9mF3ImMFf4rs1ekuQzLAb3E</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>H7bsBfYQ8BrVwWrPHqLjcN</t>
+          <t>nsNw9zroEK5eFFqvCXnWdi</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>pikowij645@coswz.com</t>
+          <t>kimocas384@1200b.com</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>qSovfnE9o9mF3ImMFf4rs1ekuQzLAb3E</t>
+          <t>ndaZlzoJCEAL2rWcFOEeuMKSrrA132tV</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>nsNw9zroEK5eFFqvCXnWdi</t>
+          <t>QM6aymxo9BHCksxvTUwwSp4</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>kimocas384@1200b.com</t>
+          <t>himir10395@1200b.com</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>ndaZlzoJCEAL2rWcFOEeuMKSrrA132tV</t>
+          <t>CQij8YQXSpkKVOXeFtwUVODsQsA7a90U</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>QM6aymxo9BHCksxvTUwwSp4</t>
+          <t>c7cz8t6G2RZKScjBvfUg7C</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>himir10395@1200b.com</t>
+          <t>xepare8732@1200b.com</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>CQij8YQXSpkKVOXeFtwUVODsQsA7a90U</t>
+          <t>3QDOjoOra9UuXpWy9msW49rTC5ST62np</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>c7cz8t6G2RZKScjBvfUg7C</t>
+          <t>aXex4ccbsE2NoxKU98uJcA</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>xepare8732@1200b.com</t>
+          <t>nikeyem927@coswz.com</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>3QDOjoOra9UuXpWy9msW49rTC5ST62np</t>
+          <t>xgVqH1xBNsc07baDwB7HbSI9oXDZ4Mbe</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>aXex4ccbsE2NoxKU98uJcA</t>
+          <t>9oXLgTF3t5eZipeHdDxkoN</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>nikeyem927@coswz.com</t>
+          <t>carom36612@coswz.com</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>xgVqH1xBNsc07baDwB7HbSI9oXDZ4Mbe</t>
+          <t>FYj1dKSpiJ8Ut1ZBkYbRmXo1pMMuxqHD</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>9oXLgTF3t5eZipeHdDxkoN</t>
+          <t>wCdZzBTZ7ZuodXp9VGrQ49</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>carom36612@coswz.com</t>
+          <t>jefico4433@1200b.com</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>FYj1dKSpiJ8Ut1ZBkYbRmXo1pMMuxqHD</t>
+          <t>Mqronv3aPXXeVMU7h4rEQ98jYqdM5Qj9</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>wCdZzBTZ7ZuodXp9VGrQ49</t>
+          <t>EniW9QPTGrEsgZjG6LsZvh</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>jefico4433@1200b.com</t>
+          <t>refok65788@1200b.com</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Mqronv3aPXXeVMU7h4rEQ98jYqdM5Qj9</t>
+          <t>HQm2YrQjWztQPeS5tcn9glppcbhJgFSt</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>EniW9QPTGrEsgZjG6LsZvh</t>
+          <t>pLgwMcrhZTMpJJhJcvTsMk</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>refok65788@1200b.com</t>
+          <t>jifol26170@1200b.com</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>HQm2YrQjWztQPeS5tcn9glppcbhJgFSt</t>
+          <t>g94mApVW76Rn8IyAUSEVwQGPPdlzJ716</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>pLgwMcrhZTMpJJhJcvTsMk</t>
+          <t>CicMLCpuGezkjGk5BRuPtN</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>jifol26170@1200b.com</t>
+          <t>benefi4649@1200b.com</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>g94mApVW76Rn8IyAUSEVwQGPPdlzJ716</t>
+          <t>GKS85X1OyHVpcXEJuYyprwl1cdFr6kF2</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>CicMLCpuGezkjGk5BRuPtN</t>
+          <t>9UhfydYnajbpbavk8CffTd</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>benefi4649@1200b.com</t>
+          <t>sopike5287@1200b.com</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>GKS85X1OyHVpcXEJuYyprwl1cdFr6kF2</t>
+          <t>mPbhTO5MojzLRb1C68gnFHwzwX7ItMw4</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>9UhfydYnajbpbavk8CffTd</t>
+          <t>Xkha5cEeszxEHfushaQdw4</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>sopike5287@1200b.com</t>
+          <t>karec14107@coswz.com</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>mPbhTO5MojzLRb1C68gnFHwzwX7ItMw4</t>
+          <t>Pev0PSY2mI6oAqhMLWS1CqkYNrw5fE8d</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Xkha5cEeszxEHfushaQdw4</t>
+          <t>EAinmt9dJmQMnyqKX7WWbE</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>karec14107@coswz.com</t>
+          <t>xavopo3145@1200b.com</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Pev0PSY2mI6oAqhMLWS1CqkYNrw5fE8d</t>
+          <t>haMuanIGVhHXeJ2MsGI7M12LJ6ZZXsaT</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>EAinmt9dJmQMnyqKX7WWbE</t>
+          <t>AQiQV2BBAz6jwafepoNqbf</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>xavopo3145@1200b.com</t>
+          <t>joriwex207@coswz.com</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>haMuanIGVhHXeJ2MsGI7M12LJ6ZZXsaT</t>
+          <t>kHUOAfblQhaESv3Jjp0IbNlEaussgW39</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>AQiQV2BBAz6jwafepoNqbf</t>
+          <t>V2csbEQ9pMFz4QUJg2jJ6i</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>joriwex207@coswz.com</t>
+          <t>voyafo9058@coswz.com</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>kHUOAfblQhaESv3Jjp0IbNlEaussgW39</t>
+          <t>FpOlWZ7m2j7npHqz1ZkT3FJ6dF0cLSxJ</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>V2csbEQ9pMFz4QUJg2jJ6i</t>
+          <t>2W2tMtPupoVuhB3oHRLJp9</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>voyafo9058@coswz.com</t>
+          <t>lexano5101@1200b.com</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>FpOlWZ7m2j7npHqz1ZkT3FJ6dF0cLSxJ</t>
+          <t>6nB2pRvb5tqXvU0CrEJx5wl3nUhgIuRv</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2W2tMtPupoVuhB3oHRLJp9</t>
+          <t>ZVYAVAPRaaXmrdPRb7ZELh</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>lexano5101@1200b.com</t>
+          <t>kirotit859@1200b.com</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>6nB2pRvb5tqXvU0CrEJx5wl3nUhgIuRv</t>
+          <t>8m6mEMsePqy6GXE49ruSBO8u1f9s0qNi</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ZVYAVAPRaaXmrdPRb7ZELh</t>
+          <t>Rb4nWVdb23evtoAQ8JrG8T</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>kirotit859@1200b.com</t>
+          <t>navet16470@1200b.com</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>8m6mEMsePqy6GXE49ruSBO8u1f9s0qNi</t>
+          <t>BMo85M8uWXIKo419Gh45BgP3QEkWemSv</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Rb4nWVdb23evtoAQ8JrG8T</t>
+          <t>beStJTkVbLtQPnJEeEHkjG</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>navet16470@1200b.com</t>
+          <t>sodeh73836@coswz.com</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>BMo85M8uWXIKo419Gh45BgP3QEkWemSv</t>
+          <t>PsVbxG4qvaLmmT8wqHmHpIqdWmCQ5d3C</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>beStJTkVbLtQPnJEeEHkjG</t>
+          <t>K6kEmvdTNsZnJBjHhMSvbP</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>sodeh73836@coswz.com</t>
+          <t>lovofes117@1200b.com</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>PsVbxG4qvaLmmT8wqHmHpIqdWmCQ5d3C</t>
+          <t>cZgYvZLIybqw9ARhD4QkpometnbkysUv</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>K6kEmvdTNsZnJBjHhMSvbP</t>
+          <t>GMMBiZmGifzYF28fSNa9c2</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>lovofes117@1200b.com</t>
+          <t>pamopi3411@1200b.com</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>cZgYvZLIybqw9ARhD4QkpometnbkysUv</t>
+          <t>PkRugnvBD3B0igMREwLPLg3sl9oeM90B</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>GMMBiZmGifzYF28fSNa9c2</t>
+          <t>UCAPmEkfidSk7cYerjyxdd</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>pamopi3411@1200b.com</t>
+          <t>jifemo1970@1200b.com</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>PkRugnvBD3B0igMREwLPLg3sl9oeM90B</t>
+          <t>imFLpCaYo6XcRqSJPCZfL11ncutZMANJ</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>UCAPmEkfidSk7cYerjyxdd</t>
+          <t>YrCYE3si4V7NcbWqAVMGCU</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>jifemo1970@1200b.com</t>
+          <t>delorow382@coswz.com</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>imFLpCaYo6XcRqSJPCZfL11ncutZMANJ</t>
+          <t>ukwJiuR0KTAlWweTSyXXnBtkyyta26Ux</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>YrCYE3si4V7NcbWqAVMGCU</t>
+          <t>BN9GkFz8CciG6LUKmXDXua</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>delorow382@coswz.com</t>
+          <t>podor68087@1200b.com</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>ukwJiuR0KTAlWweTSyXXnBtkyyta26Ux</t>
+          <t>vgsDZN5NG4tWhlactb1QcYZMGtdRQHbZ</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>BN9GkFz8CciG6LUKmXDXua</t>
+          <t>8x4oUL8G2mR6HBJFVj4XAc</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>podor68087@1200b.com</t>
+          <t>wayawa6952@coswz.com</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>vgsDZN5NG4tWhlactb1QcYZMGtdRQHbZ</t>
+          <t>oIeAeQ2KtbS65uf3b2UisJvaxPsFfi6Q</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>8x4oUL8G2mR6HBJFVj4XAc</t>
+          <t>bpeArChpJhbFCVnmZA8RJ4</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>wayawa6952@coswz.com</t>
+          <t>firav95941@1200b.com</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>oIeAeQ2KtbS65uf3b2UisJvaxPsFfi6Q</t>
+          <t>EqocVcwKEhjCDmFVeP8tFBRJ6IEZw9Hd</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>bpeArChpJhbFCVnmZA8RJ4</t>
+          <t>VqtQ6FHCbuaGK3kZ2evggF</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>firav95941@1200b.com</t>
+          <t>todel27954@1200b.com</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>EqocVcwKEhjCDmFVeP8tFBRJ6IEZw9Hd</t>
+          <t>xCOoFb986TXsBpIdSftqiOtUC4cGb47c</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>VqtQ6FHCbuaGK3kZ2evggF</t>
+          <t>Fmt2DRp7qgWkbYW2cc5cBT</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>todel27954@1200b.com</t>
+          <t>cemide9890@1200b.com</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>xCOoFb986TXsBpIdSftqiOtUC4cGb47c</t>
+          <t>xz1XAl9C6EBI0Orzw4N6MxLU4vefQ8gu</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Fmt2DRp7qgWkbYW2cc5cBT</t>
+          <t>8tm9YXNQzyNeLuUwYUJUXG</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>cemide9890@1200b.com</t>
+          <t>bohicol233@coswz.com</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>xz1XAl9C6EBI0Orzw4N6MxLU4vefQ8gu</t>
+          <t>HEIaGbLUQZL3aBgiU7DeODVxM5mzztv9</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>8tm9YXNQzyNeLuUwYUJUXG</t>
+          <t>kc7BafimJ7mQZpmfam7b8J</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>bohicol233@coswz.com</t>
+          <t>felabar963@1200b.com</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>HEIaGbLUQZL3aBgiU7DeODVxM5mzztv9</t>
+          <t>nrzMpcvs2P0JgXR56hQdwYuf4OVcAcoz</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>kc7BafimJ7mQZpmfam7b8J</t>
+          <t>9qcuYZqxJYHguQn6aAFc8P</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>felabar963@1200b.com</t>
+          <t>ritam21886@coswz.com</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>nrzMpcvs2P0JgXR56hQdwYuf4OVcAcoz</t>
+          <t>oxiBCBlg1ptibwUlGEY5t4WOGUpGuJjY</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>9qcuYZqxJYHguQn6aAFc8P</t>
+          <t>sGDP7kcxiChZc2Bx4sLPeF</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>ritam21886@coswz.com</t>
+          <t>lolama3392@coswz.com</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>oxiBCBlg1ptibwUlGEY5t4WOGUpGuJjY</t>
+          <t>EYStM48As8IXr1nfwIM4WxZ1qJUTJX2e</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>sGDP7kcxiChZc2Bx4sLPeF</t>
+          <t>ZR4i66bB2VXLrodxE99pUQ</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>lolama3392@coswz.com</t>
+          <t>yevac45467@coswz.com</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>EYStM48As8IXr1nfwIM4WxZ1qJUTJX2e</t>
+          <t>sfuWuiw2opt5IFJZ9UMJDLGqieQsLduG</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ZR4i66bB2VXLrodxE99pUQ</t>
+          <t>xkhpQ7axLsvj9WvL2eQUxW</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>yevac45467@coswz.com</t>
+          <t>wekake2133@1200b.com</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>sfuWuiw2opt5IFJZ9UMJDLGqieQsLduG</t>
+          <t>F9H7VSAxhKrx5C25wW4mtgjCHy80HG68</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>xkhpQ7axLsvj9WvL2eQUxW</t>
+          <t>tzsMtZDzfe7SiYigYvy2Lc</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>wekake2133@1200b.com</t>
+          <t>vejeme4671@coswz.com</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>F9H7VSAxhKrx5C25wW4mtgjCHy80HG68</t>
+          <t>yXXEkV1j5kwyJLZMLNiQsByYIPZ04OlS</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>tzsMtZDzfe7SiYigYvy2Lc</t>
+          <t>Z28jCiYicjtyokHCZWJrEB</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>vejeme4671@coswz.com</t>
+          <t>sivoman409@1200b.com</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>yXXEkV1j5kwyJLZMLNiQsByYIPZ04OlS</t>
+          <t>UvuMKxJ5htjJs1ok5OpPyll5RfEPiF8I</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Z28jCiYicjtyokHCZWJrEB</t>
+          <t>5FguZ3Zn6C3aB8LniffP3J</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>sivoman409@1200b.com</t>
+          <t>tejeme6947@1200b.com</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>UvuMKxJ5htjJs1ok5OpPyll5RfEPiF8I</t>
+          <t>9NRHZ5QTuYdkqyzDB4WGQFDbb9cKLdQX</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>5FguZ3Zn6C3aB8LniffP3J</t>
+          <t>SqFCfMEzZTi4KWbuHhezve</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>tejeme6947@1200b.com</t>
+          <t>yaxibos654@coswz.com</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>9NRHZ5QTuYdkqyzDB4WGQFDbb9cKLdQX</t>
+          <t>YojEjoF9kICucGwWEfRkwQ3jXntmXUb9</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>SqFCfMEzZTi4KWbuHhezve</t>
+          <t>qJc3QqXhppN7f5csRN7CJk</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>yaxibos654@coswz.com</t>
+          <t>kosiled837@1200b.com</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>YojEjoF9kICucGwWEfRkwQ3jXntmXUb9</t>
+          <t>G5PjiRNVix9C8vDatmUm41lbkBl7zADA</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>qJc3QqXhppN7f5csRN7CJk</t>
+          <t>DrdxVJAQGaCp3rH5MPcjCE</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>kosiled837@1200b.com</t>
+          <t>bejecim416@coswz.com</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>G5PjiRNVix9C8vDatmUm41lbkBl7zADA</t>
+          <t>ZK8oqUNYpic5xam0Dw3AY32KRu0YheUA</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>DrdxVJAQGaCp3rH5MPcjCE</t>
+          <t>uapU7itjAMBfJZqzh6JSoR</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>bejecim416@coswz.com</t>
+          <t>noyawer694@coswz.com</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>ZK8oqUNYpic5xam0Dw3AY32KRu0YheUA</t>
+          <t>LizuAtiXfe3CL8Trx5TvTHn4Kes47XMh</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>uapU7itjAMBfJZqzh6JSoR</t>
+          <t>9iNybNN6AYXRphPZBfiYu3</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>noyawer694@coswz.com</t>
+          <t>rawapel384@coswz.com</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>LizuAtiXfe3CL8Trx5TvTHn4Kes47XMh</t>
+          <t>YaDZvBU1AnaZj5jASC649lSTNWyx5MEd</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>9iNybNN6AYXRphPZBfiYu3</t>
+          <t>VH4wL9DJn7CJeVLxiNrsPR</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>rawapel384@coswz.com</t>
+          <t>milori7781@coswz.com</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>YaDZvBU1AnaZj5jASC649lSTNWyx5MEd</t>
+          <t>hFzcNXFLoAqcdPGmun9l7WEFqpAmEOaS</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>VH4wL9DJn7CJeVLxiNrsPR</t>
+          <t>DzVhcmiQoCj9GNGyEey8bV</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>milori7781@coswz.com</t>
+          <t>xaget22612@1200b.com</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>hFzcNXFLoAqcdPGmun9l7WEFqpAmEOaS</t>
+          <t>fQVioJODzFUzLVYuLuIh4GMtytZflRa2</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>DzVhcmiQoCj9GNGyEey8bV</t>
+          <t>hkoGzZKufWxrN2Veqi8KRF</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>xaget22612@1200b.com</t>
+          <t>lafan29114@1200b.com</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>fQVioJODzFUzLVYuLuIh4GMtytZflRa2</t>
+          <t>YFxXU1c8VvbfKyipOr8bD0YShmN7DEvR</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>hkoGzZKufWxrN2Veqi8KRF</t>
+          <t>aiRF35cN6FcH79ipXTRLXf</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>lafan29114@1200b.com</t>
+          <t>rokiji6230@1200b.com</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>YFxXU1c8VvbfKyipOr8bD0YShmN7DEvR</t>
+          <t>ygvcE5DYxeHUxkG0wLgqMpGu5T5EEUlr</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>aiRF35cN6FcH79ipXTRLXf</t>
+          <t>djbf85rvyrKiLwcLZKQWJB</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>rokiji6230@1200b.com</t>
+          <t>gajaxev858@1200b.com</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>ygvcE5DYxeHUxkG0wLgqMpGu5T5EEUlr</t>
+          <t>PzeCOI1TNljRaIjGXQ9LB6umxkv7CkXi</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>djbf85rvyrKiLwcLZKQWJB</t>
+          <t>4hTFeDdCkMpPpSwi5ZQdGD</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>gajaxev858@1200b.com</t>
+          <t>wakoxah547@coswz.com</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>PzeCOI1TNljRaIjGXQ9LB6umxkv7CkXi</t>
+          <t>XndyveOS7Kzyh7lKdJBfPE2uG8YRCMEB</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>4hTFeDdCkMpPpSwi5ZQdGD</t>
+          <t>5pJUDPketCPoLn9bg8Uw8a</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>wakoxah547@coswz.com</t>
+          <t>hekesip792@coswz.com</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>XndyveOS7Kzyh7lKdJBfPE2uG8YRCMEB</t>
+          <t>IddzLbWJBLCstiPwMcSKtPUGIRAJes7I</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>5pJUDPketCPoLn9bg8Uw8a</t>
+          <t>bE9WSksfdHYTuL7sctbf9E</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>hekesip792@coswz.com</t>
+          <t>desit76037@coswz.com</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>IddzLbWJBLCstiPwMcSKtPUGIRAJes7I</t>
+          <t>GdRWQWMORdsVhopWYKd0vkgyXhFjnEEm</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>bE9WSksfdHYTuL7sctbf9E</t>
+          <t>uSiJ39RLf2ik3RcUnewL78</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>desit76037@coswz.com</t>
+          <t>hokilo8846@coswz.com</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>GdRWQWMORdsVhopWYKd0vkgyXhFjnEEm</t>
+          <t>xy3p1a3uJzHXNrTKPBgOo8gcByWlQVbf</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>uSiJ39RLf2ik3RcUnewL78</t>
+          <t>SkV6iQWbr3uX4qAxZMqJ8e</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>hokilo8846@coswz.com</t>
+          <t>kinota3968@1200b.com</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>xy3p1a3uJzHXNrTKPBgOo8gcByWlQVbf</t>
+          <t>tVo6QytEZJhSedhbNCxuNlr6TtbDTwbG</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>SkV6iQWbr3uX4qAxZMqJ8e</t>
+          <t>GBi9PFWwb6jZvBR6tHt6tG</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>kinota3968@1200b.com</t>
+          <t>kafok91274@1200b.com</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>tVo6QytEZJhSedhbNCxuNlr6TtbDTwbG</t>
+          <t>rbSl44jvfMA0O1AgoBGn8yotnX4At9qj</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>GBi9PFWwb6jZvBR6tHt6tG</t>
+          <t>P8CJeHZPafJ9ksK4DjP9X4</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>kafok91274@1200b.com</t>
+          <t>hepivov461@coswz.com</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>rbSl44jvfMA0O1AgoBGn8yotnX4At9qj</t>
+          <t>LRWAtBvcP3OHzMNpy4pAmYoAZKt2Hzd7</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>P8CJeHZPafJ9ksK4DjP9X4</t>
+          <t>Wq2676chbay4PApch66btW</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>hepivov461@coswz.com</t>
+          <t>mediga6962@1200b.com</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>LRWAtBvcP3OHzMNpy4pAmYoAZKt2Hzd7</t>
+          <t>f5v44bGLXo945pbByUKgRRBtJrOLwV9s</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Wq2676chbay4PApch66btW</t>
+          <t>2pf6YtJVvCcCQ73GoeTwkG</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>mediga6962@1200b.com</t>
+          <t>gemesiy261@1200b.com</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>f5v44bGLXo945pbByUKgRRBtJrOLwV9s</t>
+          <t>43dDJwRPPcXgqxtpic1C8qgV5FnwTjoN</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2pf6YtJVvCcCQ73GoeTwkG</t>
+          <t>DfBW3WCK6YBxpRNpfYyFsS</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>gemesiy261@1200b.com</t>
+          <t>vopop36078@coswz.com</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>43dDJwRPPcXgqxtpic1C8qgV5FnwTjoN</t>
+          <t>ihYvMGMIiZdbtiNoT3cuAQVhOy7oai63</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>DfBW3WCK6YBxpRNpfYyFsS</t>
+          <t>JipTjAkfWuMRyWMsSHXbRT</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>vopop36078@coswz.com</t>
+          <t>liviyi2687@1200b.com</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>ihYvMGMIiZdbtiNoT3cuAQVhOy7oai63</t>
+          <t>5O8UznvS5fiwcl2Iqg0EU6LvuZfsalGa</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>JipTjAkfWuMRyWMsSHXbRT</t>
+          <t>c6MJ9qBahPoXcZnmu3LTad</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>liviyi2687@1200b.com</t>
+          <t>nojivi9674@1200b.com</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>5O8UznvS5fiwcl2Iqg0EU6LvuZfsalGa</t>
+          <t>2RhHD9yV3vccBEgtzrMnZ8Rq4HTzeh8W</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>c6MJ9qBahPoXcZnmu3LTad</t>
+          <t>ZcBcVFnKUGXyRi8xZwzpCC</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>nojivi9674@1200b.com</t>
+          <t>fixeti9021@1200b.com</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2RhHD9yV3vccBEgtzrMnZ8Rq4HTzeh8W</t>
+          <t>d7L3aNaXEKjfO4tFSBNkUVJbD8ZLNnSJ</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>ZcBcVFnKUGXyRi8xZwzpCC</t>
+          <t>qqJBK3ioMf58qe4eaurhiM</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>fixeti9021@1200b.com</t>
+          <t>widas71479@1200b.com</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>d7L3aNaXEKjfO4tFSBNkUVJbD8ZLNnSJ</t>
+          <t>55QYbQFAmv3hQrOaVpTXtNmpsU1k3dPO</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>qqJBK3ioMf58qe4eaurhiM</t>
+          <t>KVtEYD5bCvywZq65oaCDnb</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>widas71479@1200b.com</t>
+          <t>bawavip104@coswz.com</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>55QYbQFAmv3hQrOaVpTXtNmpsU1k3dPO</t>
+          <t>JtZpye7pdPl6lK7UTCMhuZoY2hvyJ9pK</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>KVtEYD5bCvywZq65oaCDnb</t>
+          <t>mTJtCxtdppM3YpyJcQDFkS</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>bawavip104@coswz.com</t>
+          <t>copawo7293@coswz.com</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>JtZpye7pdPl6lK7UTCMhuZoY2hvyJ9pK</t>
+          <t>B0Mc8vRk33LEEYPIhYNJ6GOBTsBtC7Kx</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>mTJtCxtdppM3YpyJcQDFkS</t>
+          <t>yNVgoudEmCGXPJy5TKYFuJ</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>copawo7293@coswz.com</t>
+          <t>yociko1703@1200b.com</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>B0Mc8vRk33LEEYPIhYNJ6GOBTsBtC7Kx</t>
+          <t>Uu7qo08f3qrpYeZGiovbd4b6fMvJpg5T</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>yNVgoudEmCGXPJy5TKYFuJ</t>
+          <t>w4bB4KNZafhZtw8Dv7Vq7c</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>yociko1703@1200b.com</t>
+          <t>yohiho1186@1200b.com</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Uu7qo08f3qrpYeZGiovbd4b6fMvJpg5T</t>
+          <t>y1ROvKdGD3IfK2LpQJ6emLeiryUyeTOy</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>w4bB4KNZafhZtw8Dv7Vq7c</t>
+          <t>U3eNhDLmBZ9kbbgQuTJggg</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>yohiho1186@1200b.com</t>
+          <t>vepek51758@coswz.com</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>y1ROvKdGD3IfK2LpQJ6emLeiryUyeTOy</t>
+          <t>Xd0XnvFWpuYJb6EyX4v0qZGJyzKPbpjf</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>U3eNhDLmBZ9kbbgQuTJggg</t>
+          <t>K7wD42ADsf3yKih2DpdZX3</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>vepek51758@coswz.com</t>
+          <t>vicexa9591@coswz.com</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Xd0XnvFWpuYJb6EyX4v0qZGJyzKPbpjf</t>
+          <t>npz20JjzNH92wIH4tCQx49nC0it14Xxw</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>K7wD42ADsf3yKih2DpdZX3</t>
+          <t>rZd7CALt2MZEMHmpDtGQxB</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>vicexa9591@coswz.com</t>
+          <t>hecab14854@1200b.com</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>npz20JjzNH92wIH4tCQx49nC0it14Xxw</t>
+          <t>K8wwgIDz5G56KxRoP7JgMK2PO7C2UzvN</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>rZd7CALt2MZEMHmpDtGQxB</t>
+          <t>4KT5DztHkEUnCgYrNhRx4e</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>hecab14854@1200b.com</t>
+          <t>carexan555@coswz.com</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>K8wwgIDz5G56KxRoP7JgMK2PO7C2UzvN</t>
+          <t>cBLSH97sWXVnfO4kUKBNbM8eYNZcanHx</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>4KT5DztHkEUnCgYrNhRx4e</t>
+          <t>HW37WS2fucmm8m6ZUSMU7Q</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>carexan555@coswz.com</t>
+          <t>lokos77574@coswz.com</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>cBLSH97sWXVnfO4kUKBNbM8eYNZcanHx</t>
+          <t>rNU7s0xkwJcc3DDFI9osfwRqVJB5MUvd</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>HW37WS2fucmm8m6ZUSMU7Q</t>
+          <t>777awg7nDxL7oVL4duMc6h</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>lokos77574@coswz.com</t>
+          <t>nojex76241@1200b.com</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>rNU7s0xkwJcc3DDFI9osfwRqVJB5MUvd</t>
+          <t>Kz7OdwkMZTZaDJQ1iUTZLbGvoS84keOP</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>777awg7nDxL7oVL4duMc6h</t>
+          <t>hVpkXzmpNbzDE5fFtiJbc2</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>nojex76241@1200b.com</t>
+          <t>hovifim988@1200b.com</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Kz7OdwkMZTZaDJQ1iUTZLbGvoS84keOP</t>
+          <t>CK0Wp6WKiFD7acjl10G8vysxWR48wZRg</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>hVpkXzmpNbzDE5fFtiJbc2</t>
+          <t>P5XJ2dTaNUHsMkCoMgVS8i</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>hovifim988@1200b.com</t>
+          <t>yawoc12567@coswz.com</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>CK0Wp6WKiFD7acjl10G8vysxWR48wZRg</t>
+          <t>uT6UL7Qo9WWZFIw6nFihvEoPsRuWB2cB</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>P5XJ2dTaNUHsMkCoMgVS8i</t>
+          <t>J8JUeTV2yxn9wmuA5vLnfW</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>yawoc12567@coswz.com</t>
+          <t>gecadac197@coswz.com</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>uT6UL7Qo9WWZFIw6nFihvEoPsRuWB2cB</t>
+          <t>Grzwxyx41AkWP5m4f3xtEu0JlfrFim7P</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>J8JUeTV2yxn9wmuA5vLnfW</t>
+          <t>SARbUSMkNZD9XjpwUeK4oH</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>gecadac197@coswz.com</t>
+          <t>goyixov775@1200b.com</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Grzwxyx41AkWP5m4f3xtEu0JlfrFim7P</t>
+          <t>h6VvXzCUwwTE11bRqNCZS8brKBY5zCbz</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>SARbUSMkNZD9XjpwUeK4oH</t>
+          <t>REZRkCf7tSD37FJmyWRET3</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>goyixov775@1200b.com</t>
+          <t>jayit97735@1200b.com</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>h6VvXzCUwwTE11bRqNCZS8brKBY5zCbz</t>
+          <t>xstn0Y1QeBj5bnDGrXeOn648TCmCcc0G</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>REZRkCf7tSD37FJmyWRET3</t>
+          <t>9LJtRkXV4MTjAwMVwgoUaf</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>jayit97735@1200b.com</t>
+          <t>tiyeciy866@1200b.com</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>xstn0Y1QeBj5bnDGrXeOn648TCmCcc0G</t>
+          <t>3P4jyDaUqq5fdNqWDIb34rlZbRf2KCxG</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>9LJtRkXV4MTjAwMVwgoUaf</t>
+          <t>RSr7tgrfTd94Mm3owU2Ry3</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>tiyeciy866@1200b.com</t>
+          <t>racek36029@1200b.com</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>3P4jyDaUqq5fdNqWDIb34rlZbRf2KCxG</t>
+          <t>hDghGPPIJ1UDWE5TaZJEOsOhg3DQYHkJ</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>RSr7tgrfTd94Mm3owU2Ry3</t>
+          <t>V3rPPRdJNBBWxdp37MKNZg</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>racek36029@1200b.com</t>
+          <t>lenac61027@coswz.com</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>hDghGPPIJ1UDWE5TaZJEOsOhg3DQYHkJ</t>
+          <t>xCgpDNXZ0OxWUZTv3cCs15Fx5gcmbGih</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
-        <is>
-          <t>V3rPPRdJNBBWxdp37MKNZg</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="inlineStr">
-        <is>
-          <t>lenac61027@coswz.com</t>
-        </is>
-      </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>xCgpDNXZ0OxWUZTv3cCs15Fx5gcmbGih</t>
-        </is>
-      </c>
-      <c r="C165" t="inlineStr">
         <is>
           <t>JrV6Aq9rfLw9W5Kf8jPry4</t>
         </is>

</xml_diff>